<commit_message>
working decrement for inventory in heuristic
</commit_message>
<xml_diff>
--- a/L-shaped/Final_codes/data/Starting_point.xlsx
+++ b/L-shaped/Final_codes/data/Starting_point.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fthcn\Desktop\Vaccine_Tender_Scheduling_Problem\Julia_Files\L-shaped method\Using_deterministic_model_from_IISE_paper\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/L-shaped/Final_codes/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{E4667220-B6D3-44CA-BB2C-7EE709A98D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D97F6FD3-B23A-4A36-A445-5D1855D05295}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13550" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="F_start" sheetId="2" r:id="rId1"/>
@@ -557,9 +557,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{942AD6D9-E2BE-4540-AD66-B6783F716305}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>38</v>
       </c>
@@ -570,7 +574,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -581,7 +585,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -592,7 +596,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -603,7 +607,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -614,7 +618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -625,7 +629,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -636,7 +640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -647,7 +651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
@@ -658,7 +662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -669,7 +673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -680,7 +684,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -691,7 +695,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -711,15 +715,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E851515-DB43-462D-9C92-F50748C0A12A}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:E27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="8.85546875" style="2"/>
     <col min="2" max="2" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="8.88671875" style="2"/>
-    <col min="5" max="5" width="16.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="8.85546875" style="2"/>
+    <col min="5" max="5" width="16.140625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>14</v>
       </c>
@@ -736,7 +740,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
@@ -753,7 +757,7 @@
         <v>13299</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>21</v>
       </c>
@@ -770,7 +774,7 @@
         <v>12505</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>21</v>
       </c>
@@ -787,7 +791,7 @@
         <v>13547</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
@@ -804,7 +808,7 @@
         <v>6547</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
@@ -821,7 +825,7 @@
         <v>90279</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>27</v>
       </c>
@@ -838,7 +842,7 @@
         <v>180177</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>27</v>
       </c>
@@ -855,7 +859,7 @@
         <v>13305</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>29</v>
       </c>
@@ -872,7 +876,7 @@
         <v>8948</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>29</v>
       </c>
@@ -889,7 +893,7 @@
         <v>140932</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>29</v>
       </c>
@@ -906,7 +910,7 @@
         <v>17896</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>29</v>
       </c>
@@ -923,7 +927,7 @@
         <v>31318</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>29</v>
       </c>
@@ -940,7 +944,7 @@
         <v>53688</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
@@ -957,7 +961,7 @@
         <v>43365</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>32</v>
       </c>
@@ -974,7 +978,7 @@
         <v>40214</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>34</v>
       </c>
@@ -991,7 +995,7 @@
         <v>219201</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>34</v>
       </c>
@@ -1008,7 +1012,7 @@
         <v>61221</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>34</v>
       </c>
@@ -1025,7 +1029,7 @@
         <v>84681</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>9</v>
       </c>
@@ -1042,7 +1046,7 @@
         <v>3625</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
@@ -1059,7 +1063,7 @@
         <v>13464</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>9</v>
       </c>
@@ -1076,7 +1080,7 @@
         <v>5391</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>10</v>
       </c>
@@ -1093,7 +1097,7 @@
         <v>56510</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>10</v>
       </c>
@@ -1110,7 +1114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>10</v>
       </c>
@@ -1127,7 +1131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>13</v>
       </c>
@@ -1144,7 +1148,7 @@
         <v>185663</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>13</v>
       </c>
@@ -1161,7 +1165,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>13</v>
       </c>
@@ -1187,13 +1191,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AF8CA8F-1DBE-42B3-8633-48C2ED5062E9}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>14</v>
       </c>
@@ -1201,7 +1205,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -1209,7 +1213,7 @@
         <v>137010500</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -1217,7 +1221,7 @@
         <v>283717500</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -1225,7 +1229,7 @@
         <v>9879500</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1233,7 +1237,7 @@
         <v>108804000</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1241,7 +1245,7 @@
         <v>46674000</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -1249,7 +1253,7 @@
         <v>143467000</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1257,7 +1261,7 @@
         <v>11463500</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>39</v>
       </c>
@@ -1265,7 +1269,7 @@
         <v>10000000</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>40</v>
       </c>
@@ -1273,7 +1277,7 @@
         <v>10000000</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>7</v>
       </c>
@@ -1281,7 +1285,7 @@
         <v>10000000</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>41</v>
       </c>
@@ -1289,7 +1293,7 @@
         <v>10000000</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>27</v>
       </c>
@@ -1297,7 +1301,7 @@
         <v>143856000</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>42</v>
       </c>
@@ -1305,7 +1309,7 @@
         <v>10000000</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>43</v>
       </c>
@@ -1313,7 +1317,7 @@
         <v>10000000</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>44</v>
       </c>
@@ -1321,7 +1325,7 @@
         <v>43714500</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>9</v>
       </c>
@@ -1329,7 +1333,7 @@
         <v>9216211.8592507206</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>10</v>
       </c>
@@ -1346,13 +1350,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{903BEB0C-00BA-4B81-9CB6-933B54D27020}">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.6640625" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>45</v>
       </c>
@@ -1360,7 +1364,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1368,7 +1372,7 @@
         <v>109769715.256769</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1376,7 +1380,7 @@
         <v>76483381.4640522</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1384,7 +1388,7 @@
         <v>111936141.058823</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -1392,7 +1396,7 @@
         <v>6763202.4705882296</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -1400,7 +1404,7 @@
         <v>50081880.540420704</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1408,7 +1412,7 @@
         <v>59034355.4808589</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1416,7 +1420,7 @@
         <v>171888397.557423</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -1424,7 +1428,7 @@
         <v>52857961.247619003</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
@@ -1432,7 +1436,7 @@
         <v>63880730.2712842</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1440,7 +1444,7 @@
         <v>106632842.278244</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -1448,7 +1452,7 @@
         <v>148000000</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>

</xml_diff>